<commit_message>
Cambios en las ressitencias R15 y R20 a 10Ohm
</commit_message>
<xml_diff>
--- a/02.HARDWARE/V2-ROVER R-1/02.BOM/BATT_DCDC.xlsx
+++ b/02.HARDWARE/V2-ROVER R-1/02.BOM/BATT_DCDC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Team Dropbox\JRODRIGUEZ\Repositorios\01.Rover\02.HARDWARE\V2-ROVER R-1\02.BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B48828-3482-486B-98DF-C2456BAF78A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FFD7611-D407-47CC-80DA-79A027D20764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BATT_DCDC" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="159">
   <si>
     <t>Qty</t>
   </si>
@@ -506,9 +506,6 @@
     <t>R15, R20</t>
   </si>
   <si>
-    <t>20R</t>
-  </si>
-  <si>
     <t>R5, R19</t>
   </si>
   <si>
@@ -524,6 +521,12 @@
   </si>
   <si>
     <t>NO MONTAR</t>
+  </si>
+  <si>
+    <t>10R</t>
+  </si>
+  <si>
+    <t>Se cambia el valor de la posicion 42 de 20R a 10R.</t>
   </si>
 </sst>
 </file>
@@ -1449,9 +1452,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1489,7 +1492,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1595,7 +1598,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1737,7 +1740,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1770,7 +1773,7 @@
       </c>
       <c r="B2" s="3">
         <f>MAX(_HISTORY!A4:A55)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" s="25"/>
     </row>
@@ -1809,7 +1812,7 @@
         <v>71</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>0</v>
@@ -2489,7 +2492,7 @@
         <v>2</v>
       </c>
       <c r="E32" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F32" t="s">
         <v>20</v>
@@ -2883,7 +2886,7 @@
         <v>150</v>
       </c>
       <c r="L47" s="20" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2894,7 +2897,7 @@
         <v>134</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D48">
         <v>2</v>
@@ -2903,7 +2906,7 @@
         <v>151</v>
       </c>
       <c r="F48" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="G48" t="s">
         <v>60</v>
@@ -2950,7 +2953,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5396D425-0A04-B64D-B9F7-D3F9797B3C5D}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="4" max="4" width="55.85546875" style="19" customWidth="1"/>
@@ -3112,7 +3115,21 @@
         <v>87</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>154</v>
+        <v>153</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14">
+        <v>11</v>
+      </c>
+      <c r="B14" s="22">
+        <v>45411</v>
+      </c>
+      <c r="C14" t="s">
+        <v>87</v>
+      </c>
+      <c r="D14" s="19" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add C11 y R22.
</commit_message>
<xml_diff>
--- a/02.HARDWARE/V2-ROVER R-1/02.BOM/BATT_DCDC.xlsx
+++ b/02.HARDWARE/V2-ROVER R-1/02.BOM/BATT_DCDC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Team Dropbox\JRODRIGUEZ\Repositorios\01.Rover\02.HARDWARE\V2-ROVER R-1\02.BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37FC938C-0E93-41CD-8B1D-3D5DE38DAD55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96D9637D-5AC1-4BDA-8F62-583809AC8421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BATT_DCDC" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="157">
   <si>
     <t>Document property of:</t>
   </si>
@@ -221,9 +221,6 @@
     <t>47uF 25V</t>
   </si>
   <si>
-    <t>C2, C5, C6,C8 C24</t>
-  </si>
-  <si>
     <t>100nF, 25V, X7R o X5R</t>
   </si>
   <si>
@@ -452,9 +449,6 @@
     <t>N.A</t>
   </si>
   <si>
-    <t>R7,R21</t>
-  </si>
-  <si>
     <t>4k3</t>
   </si>
   <si>
@@ -522,6 +516,16 @@
   </si>
   <si>
     <t>20R</t>
+  </si>
+  <si>
+    <t>R7,R21,R22</t>
+  </si>
+  <si>
+    <t>C2, C5, C6,C8 C24,C11</t>
+  </si>
+  <si>
+    <t>Se añade a la posicion 35 el part R22 se cambia la cantidad de 2 a 3
+Se añade a la posicion 5 el part C11 se cambia la cantidad de 5 a 6</t>
   </si>
 </sst>
 </file>
@@ -871,9 +875,6 @@
     <xf numFmtId="14" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -957,12 +958,19 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -980,7 +988,7 @@
   <autoFilter ref="A6:L48" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Position"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="NEW"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="NEW" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Assembly"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Qty"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Part"/>
@@ -1287,10 +1295,10 @@
   <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" style="22" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" style="42" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5703125" style="43" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" style="22" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" style="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" style="41" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" style="42" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" style="21" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="30.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="20.85546875" bestFit="1" customWidth="1"/>
@@ -1301,82 +1309,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="18.75" customHeight="1">
-      <c r="B1" s="23"/>
-      <c r="C1" s="24"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="23"/>
     </row>
     <row r="2" spans="1:12" ht="20.25" customHeight="1">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="26">
+      <c r="B2" s="25">
         <f>MAX(_HISTORY!A4:A55)</f>
-        <v>12</v>
-      </c>
-      <c r="C2" s="27"/>
+        <v>13</v>
+      </c>
+      <c r="C2" s="26"/>
     </row>
     <row r="3" spans="1:12" ht="29.25" customHeight="1">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="28">
-        <f>VLOOKUP(B2,_HISTORY!A3:D15,2)</f>
-        <v>45545</v>
-      </c>
-      <c r="C3" s="28"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="30"/>
+      <c r="B3" s="27">
+        <f>VLOOKUP(B2,_HISTORY!A3:D100,2)</f>
+        <v>45553</v>
+      </c>
+      <c r="C3" s="27"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="29"/>
     </row>
     <row r="4" spans="1:12" ht="30" customHeight="1">
-      <c r="B4" s="44" t="s">
+      <c r="B4" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="45"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="47"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="44"/>
+      <c r="F4" s="46"/>
     </row>
     <row r="5" spans="1:12" ht="30.75" customHeight="1">
-      <c r="B5" s="31"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="34"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="33"/>
     </row>
     <row r="6" spans="1:12" ht="18.75" customHeight="1">
-      <c r="A6" s="35" t="s">
+      <c r="A6" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="37" t="s">
+      <c r="C6" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="35" t="s">
+      <c r="D6" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="37" t="s">
+      <c r="E6" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="37" t="s">
+      <c r="F6" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="G6" s="37" t="s">
+      <c r="G6" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="H6" s="37" t="s">
+      <c r="H6" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="I6" s="37" t="s">
+      <c r="I6" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="J6" s="37" t="s">
+      <c r="J6" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="K6" s="37" t="s">
+      <c r="K6" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="L6" s="37" t="s">
+      <c r="L6" s="36" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1384,10 +1392,10 @@
       <c r="A7" s="17">
         <v>1</v>
       </c>
-      <c r="B7" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C7" s="24"/>
+      <c r="B7" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="23"/>
       <c r="D7" s="17">
         <v>2</v>
       </c>
@@ -1408,10 +1416,10 @@
       <c r="A8" s="17">
         <v>2</v>
       </c>
-      <c r="B8" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" s="24"/>
+      <c r="B8" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="23"/>
       <c r="D8" s="17">
         <v>2</v>
       </c>
@@ -1432,10 +1440,10 @@
       <c r="A9" s="17">
         <v>3</v>
       </c>
-      <c r="B9" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" s="24"/>
+      <c r="B9" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="23"/>
       <c r="D9" s="17">
         <v>2</v>
       </c>
@@ -1456,10 +1464,10 @@
       <c r="A10" s="17">
         <v>4</v>
       </c>
-      <c r="B10" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="24"/>
+      <c r="B10" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="23"/>
       <c r="D10" s="17">
         <v>2</v>
       </c>
@@ -1480,18 +1488,18 @@
       <c r="A11" s="17">
         <v>5</v>
       </c>
-      <c r="B11" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" s="24"/>
+      <c r="B11" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="C11" s="23"/>
       <c r="D11" s="17">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E11" t="s">
+        <v>155</v>
+      </c>
+      <c r="F11" t="s">
         <v>55</v>
-      </c>
-      <c r="F11" t="s">
-        <v>56</v>
       </c>
       <c r="G11" t="s">
         <v>45</v>
@@ -1501,55 +1509,55 @@
       </c>
     </row>
     <row r="12" spans="1:12" ht="18.75" customHeight="1">
-      <c r="A12" s="38">
+      <c r="A12" s="37">
         <v>6</v>
       </c>
-      <c r="B12" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" s="39"/>
-      <c r="D12" s="40" t="s">
-        <v>57</v>
-      </c>
-      <c r="E12" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="F12" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="G12" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="H12" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="I12" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="J12" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="K12" s="39"/>
-      <c r="L12" s="39" t="s">
-        <v>57</v>
+      <c r="B12" s="49" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="38"/>
+      <c r="D12" s="39" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="G12" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="H12" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="I12" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="J12" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="K12" s="38"/>
+      <c r="L12" s="38" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="18.75" customHeight="1">
       <c r="A13" s="17">
         <v>7</v>
       </c>
-      <c r="B13" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C13" s="24"/>
+      <c r="B13" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="23"/>
       <c r="D13" s="17">
         <v>1</v>
       </c>
       <c r="E13" t="s">
+        <v>57</v>
+      </c>
+      <c r="F13" t="s">
         <v>58</v>
-      </c>
-      <c r="F13" t="s">
-        <v>59</v>
       </c>
       <c r="G13" t="s">
         <v>45</v>
@@ -1559,278 +1567,278 @@
       </c>
     </row>
     <row r="14" spans="1:12" ht="18.75" customHeight="1">
-      <c r="A14" s="38">
+      <c r="A14" s="37">
         <v>8</v>
       </c>
-      <c r="B14" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" s="39"/>
-      <c r="D14" s="40" t="s">
-        <v>57</v>
-      </c>
-      <c r="E14" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="F14" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="G14" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="H14" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="I14" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="J14" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="K14" s="39"/>
-      <c r="L14" s="39" t="s">
-        <v>57</v>
+      <c r="B14" s="49" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="38"/>
+      <c r="D14" s="39" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="F14" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="G14" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="H14" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="I14" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="J14" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="K14" s="38"/>
+      <c r="L14" s="38" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="18.75" customHeight="1">
       <c r="A15" s="17">
         <v>9</v>
       </c>
-      <c r="B15" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C15" s="24"/>
+      <c r="B15" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="23"/>
       <c r="D15" s="17">
         <v>1</v>
       </c>
       <c r="E15" t="s">
+        <v>59</v>
+      </c>
+      <c r="F15" t="s">
         <v>60</v>
-      </c>
-      <c r="F15" t="s">
-        <v>61</v>
       </c>
       <c r="G15" t="s">
         <v>45</v>
       </c>
       <c r="H15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="19.5" customHeight="1">
       <c r="A16" s="17">
         <v>10</v>
       </c>
-      <c r="B16" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" s="24"/>
+      <c r="B16" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="23"/>
       <c r="D16" s="17">
         <v>1</v>
       </c>
       <c r="E16" t="s">
+        <v>62</v>
+      </c>
+      <c r="F16" t="s">
         <v>63</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>64</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>65</v>
-      </c>
-      <c r="H16" t="s">
-        <v>66</v>
       </c>
       <c r="K16" s="5"/>
       <c r="L16" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="19.5" customHeight="1">
       <c r="A17" s="17">
         <v>11</v>
       </c>
-      <c r="B17" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C17" s="24"/>
+      <c r="B17" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="23"/>
       <c r="D17" s="17">
         <v>1</v>
       </c>
       <c r="E17" t="s">
+        <v>67</v>
+      </c>
+      <c r="F17" t="s">
         <v>68</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
+        <v>64</v>
+      </c>
+      <c r="H17" t="s">
         <v>69</v>
-      </c>
-      <c r="G17" t="s">
-        <v>65</v>
-      </c>
-      <c r="H17" t="s">
-        <v>70</v>
       </c>
       <c r="K17" s="5"/>
       <c r="L17" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="19.5" customHeight="1">
       <c r="A18" s="17">
         <v>12</v>
       </c>
-      <c r="B18" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C18" s="24"/>
+      <c r="B18" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C18" s="23"/>
       <c r="D18" s="17">
         <v>1</v>
       </c>
       <c r="E18" t="s">
+        <v>71</v>
+      </c>
+      <c r="F18" t="s">
         <v>72</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>73</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>74</v>
-      </c>
-      <c r="H18" t="s">
-        <v>75</v>
       </c>
       <c r="K18" s="5"/>
       <c r="L18" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="19.5" customHeight="1">
       <c r="A19" s="17">
         <v>13</v>
       </c>
-      <c r="B19" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C19" s="24"/>
+      <c r="B19" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" s="23"/>
       <c r="D19" s="17">
         <v>1</v>
       </c>
       <c r="E19" t="s">
+        <v>76</v>
+      </c>
+      <c r="F19" t="s">
         <v>77</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>78</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>79</v>
       </c>
-      <c r="H19" t="s">
+      <c r="K19" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="K19" s="5" t="s">
+      <c r="L19" s="5" t="s">
         <v>81</v>
-      </c>
-      <c r="L19" s="5" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="18.75" customHeight="1">
       <c r="A20" s="17">
         <v>14</v>
       </c>
-      <c r="B20" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C20" s="24"/>
+      <c r="B20" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="23"/>
       <c r="D20" s="17">
         <v>1</v>
       </c>
       <c r="E20" t="s">
+        <v>82</v>
+      </c>
+      <c r="F20" t="s">
         <v>83</v>
       </c>
-      <c r="F20" t="s">
-        <v>84</v>
-      </c>
       <c r="G20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="18.75" customHeight="1">
       <c r="A21" s="17">
         <v>15</v>
       </c>
-      <c r="B21" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C21" s="24"/>
+      <c r="B21" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="23"/>
       <c r="D21" s="17">
         <v>1</v>
       </c>
       <c r="E21" t="s">
+        <v>84</v>
+      </c>
+      <c r="F21" t="s">
         <v>85</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>86</v>
-      </c>
-      <c r="G21" t="s">
-        <v>87</v>
       </c>
       <c r="H21" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="18.75" customHeight="1">
-      <c r="A22" s="38">
+      <c r="A22" s="37">
         <v>16</v>
       </c>
-      <c r="B22" s="23" t="s">
-        <v>88</v>
-      </c>
-      <c r="C22" s="39"/>
-      <c r="D22" s="40" t="s">
-        <v>57</v>
-      </c>
-      <c r="E22" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="F22" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="G22" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="H22" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="I22" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="J22" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="K22" s="39"/>
-      <c r="L22" s="39" t="s">
-        <v>57</v>
+      <c r="B22" s="49" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" s="38"/>
+      <c r="D22" s="39" t="s">
+        <v>56</v>
+      </c>
+      <c r="E22" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="F22" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="G22" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="H22" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="I22" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="J22" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="K22" s="38"/>
+      <c r="L22" s="38" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="23" spans="1:12" ht="18.75" customHeight="1">
       <c r="A23" s="17">
         <v>17</v>
       </c>
-      <c r="B23" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C23" s="24"/>
+      <c r="B23" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" s="23"/>
       <c r="D23" s="17">
         <v>1</v>
       </c>
       <c r="E23" t="s">
+        <v>88</v>
+      </c>
+      <c r="F23" t="s">
         <v>89</v>
       </c>
-      <c r="F23" t="s">
-        <v>90</v>
-      </c>
       <c r="G23" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H23" t="s">
         <v>46</v>
@@ -1840,21 +1848,21 @@
       <c r="A24" s="17">
         <v>18</v>
       </c>
-      <c r="B24" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C24" s="24"/>
+      <c r="B24" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" s="23"/>
       <c r="D24" s="17">
         <v>1</v>
       </c>
       <c r="E24" t="s">
+        <v>90</v>
+      </c>
+      <c r="F24" t="s">
         <v>91</v>
       </c>
-      <c r="F24" t="s">
-        <v>92</v>
-      </c>
       <c r="G24" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H24" t="s">
         <v>46</v>
@@ -1864,21 +1872,21 @@
       <c r="A25" s="17">
         <v>19</v>
       </c>
-      <c r="B25" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C25" s="24"/>
+      <c r="B25" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="23"/>
       <c r="D25" s="17">
         <v>1</v>
       </c>
       <c r="E25" t="s">
+        <v>92</v>
+      </c>
+      <c r="F25" t="s">
         <v>93</v>
       </c>
-      <c r="F25" t="s">
-        <v>94</v>
-      </c>
       <c r="G25" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H25" t="s">
         <v>46</v>
@@ -1888,21 +1896,21 @@
       <c r="A26" s="17">
         <v>20</v>
       </c>
-      <c r="B26" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C26" s="24"/>
+      <c r="B26" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" s="23"/>
       <c r="D26" s="17">
         <v>1</v>
       </c>
       <c r="E26" t="s">
+        <v>94</v>
+      </c>
+      <c r="F26" t="s">
         <v>95</v>
       </c>
-      <c r="F26" t="s">
-        <v>96</v>
-      </c>
       <c r="G26" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H26" t="s">
         <v>46</v>
@@ -1912,21 +1920,21 @@
       <c r="A27" s="17">
         <v>21</v>
       </c>
-      <c r="B27" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C27" s="24"/>
+      <c r="B27" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C27" s="23"/>
       <c r="D27" s="17">
         <v>1</v>
       </c>
       <c r="E27" t="s">
+        <v>96</v>
+      </c>
+      <c r="F27" t="s">
         <v>97</v>
       </c>
-      <c r="F27" t="s">
-        <v>98</v>
-      </c>
       <c r="G27" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H27" t="s">
         <v>49</v>
@@ -1936,21 +1944,21 @@
       <c r="A28" s="17">
         <v>22</v>
       </c>
-      <c r="B28" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C28" s="24"/>
+      <c r="B28" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C28" s="23"/>
       <c r="D28" s="17">
         <v>2</v>
       </c>
       <c r="E28" t="s">
+        <v>98</v>
+      </c>
+      <c r="F28" t="s">
         <v>99</v>
       </c>
-      <c r="F28" t="s">
-        <v>100</v>
-      </c>
       <c r="G28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H28" t="s">
         <v>46</v>
@@ -1960,21 +1968,21 @@
       <c r="A29" s="17">
         <v>23</v>
       </c>
-      <c r="B29" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C29" s="24"/>
+      <c r="B29" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C29" s="23"/>
       <c r="D29" s="17">
         <v>1</v>
       </c>
       <c r="E29" t="s">
+        <v>100</v>
+      </c>
+      <c r="F29" t="s">
         <v>101</v>
       </c>
-      <c r="F29" t="s">
-        <v>102</v>
-      </c>
       <c r="G29" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H29" t="s">
         <v>46</v>
@@ -1984,21 +1992,21 @@
       <c r="A30" s="17">
         <v>24</v>
       </c>
-      <c r="B30" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C30" s="24"/>
+      <c r="B30" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C30" s="23"/>
       <c r="D30" s="17">
         <v>1</v>
       </c>
       <c r="E30" t="s">
+        <v>102</v>
+      </c>
+      <c r="F30" t="s">
         <v>103</v>
       </c>
-      <c r="F30" t="s">
-        <v>104</v>
-      </c>
       <c r="G30" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H30" t="s">
         <v>46</v>
@@ -2008,21 +2016,21 @@
       <c r="A31" s="17">
         <v>25</v>
       </c>
-      <c r="B31" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C31" s="24"/>
+      <c r="B31" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C31" s="23"/>
       <c r="D31" s="17">
         <v>1</v>
       </c>
       <c r="E31" t="s">
+        <v>104</v>
+      </c>
+      <c r="F31" t="s">
         <v>105</v>
       </c>
-      <c r="F31" t="s">
-        <v>106</v>
-      </c>
       <c r="G31" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H31" t="s">
         <v>46</v>
@@ -2032,21 +2040,21 @@
       <c r="A32" s="17">
         <v>26</v>
       </c>
-      <c r="B32" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C32" s="24"/>
+      <c r="B32" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C32" s="23"/>
       <c r="D32" s="17">
         <v>2</v>
       </c>
       <c r="E32" t="s">
+        <v>106</v>
+      </c>
+      <c r="F32" t="s">
         <v>107</v>
       </c>
-      <c r="F32" t="s">
-        <v>108</v>
-      </c>
       <c r="G32" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H32" t="s">
         <v>46</v>
@@ -2056,21 +2064,21 @@
       <c r="A33" s="17">
         <v>27</v>
       </c>
-      <c r="B33" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C33" s="24"/>
+      <c r="B33" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C33" s="23"/>
       <c r="D33" s="17">
         <v>1</v>
       </c>
       <c r="E33" t="s">
+        <v>108</v>
+      </c>
+      <c r="F33" t="s">
         <v>109</v>
       </c>
-      <c r="F33" t="s">
-        <v>110</v>
-      </c>
       <c r="G33" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H33" t="s">
         <v>49</v>
@@ -2080,21 +2088,21 @@
       <c r="A34" s="17">
         <v>28</v>
       </c>
-      <c r="B34" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C34" s="24"/>
+      <c r="B34" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C34" s="23"/>
       <c r="D34" s="17">
         <v>1</v>
       </c>
       <c r="E34" t="s">
+        <v>110</v>
+      </c>
+      <c r="F34" t="s">
         <v>111</v>
       </c>
-      <c r="F34" t="s">
-        <v>112</v>
-      </c>
       <c r="G34" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H34" t="s">
         <v>49</v>
@@ -2104,21 +2112,21 @@
       <c r="A35" s="17">
         <v>29</v>
       </c>
-      <c r="B35" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C35" s="24"/>
+      <c r="B35" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C35" s="23"/>
       <c r="D35" s="17">
         <v>1</v>
       </c>
       <c r="E35" t="s">
+        <v>112</v>
+      </c>
+      <c r="F35" t="s">
         <v>113</v>
       </c>
-      <c r="F35" t="s">
-        <v>114</v>
-      </c>
       <c r="G35" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H35" t="s">
         <v>46</v>
@@ -2128,102 +2136,102 @@
       <c r="A36" s="17">
         <v>30</v>
       </c>
-      <c r="B36" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C36" s="24"/>
+      <c r="B36" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C36" s="23"/>
       <c r="D36" s="17">
         <v>1</v>
       </c>
       <c r="E36" t="s">
+        <v>114</v>
+      </c>
+      <c r="F36" t="s">
         <v>115</v>
       </c>
-      <c r="F36" t="s">
+      <c r="G36" t="s">
+        <v>86</v>
+      </c>
+      <c r="H36" t="s">
         <v>116</v>
-      </c>
-      <c r="G36" t="s">
-        <v>87</v>
-      </c>
-      <c r="H36" t="s">
-        <v>117</v>
       </c>
       <c r="K36" s="5"/>
       <c r="L36" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="37" spans="1:12" ht="18.75" customHeight="1">
       <c r="A37" s="17">
         <v>31</v>
       </c>
-      <c r="B37" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C37" s="24"/>
+      <c r="B37" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C37" s="23"/>
       <c r="D37" s="17">
         <v>2</v>
       </c>
       <c r="E37" t="s">
+        <v>118</v>
+      </c>
+      <c r="F37" t="s">
         <v>119</v>
       </c>
-      <c r="F37" t="s">
+      <c r="G37" t="s">
         <v>120</v>
       </c>
-      <c r="G37" t="s">
+      <c r="H37" t="s">
         <v>121</v>
-      </c>
-      <c r="H37" t="s">
-        <v>122</v>
       </c>
       <c r="K37" s="5"/>
       <c r="L37" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="38" spans="1:12" ht="18.75" customHeight="1">
       <c r="A38" s="17">
         <v>32</v>
       </c>
-      <c r="B38" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C38" s="24"/>
+      <c r="B38" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C38" s="23"/>
       <c r="D38" s="17">
         <v>1</v>
       </c>
       <c r="E38" t="s">
+        <v>123</v>
+      </c>
+      <c r="F38" t="s">
         <v>124</v>
       </c>
-      <c r="F38" t="s">
+      <c r="G38" t="s">
+        <v>120</v>
+      </c>
+      <c r="H38" t="s">
         <v>125</v>
-      </c>
-      <c r="G38" t="s">
-        <v>121</v>
-      </c>
-      <c r="H38" t="s">
-        <v>126</v>
       </c>
       <c r="K38" s="5"/>
       <c r="L38" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="39" spans="1:12" ht="18.75" customHeight="1">
       <c r="A39" s="17">
         <v>33</v>
       </c>
-      <c r="B39" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C39" s="24"/>
+      <c r="B39" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C39" s="23"/>
       <c r="D39" s="17">
         <v>1</v>
       </c>
       <c r="E39" t="s">
+        <v>127</v>
+      </c>
+      <c r="F39" t="s">
         <v>128</v>
-      </c>
-      <c r="F39" t="s">
-        <v>129</v>
       </c>
       <c r="G39" t="s">
         <v>45</v>
@@ -2236,18 +2244,18 @@
       <c r="A40" s="17">
         <v>34</v>
       </c>
-      <c r="B40" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C40" s="24"/>
+      <c r="B40" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C40" s="23"/>
       <c r="D40" s="17">
         <v>1</v>
       </c>
       <c r="E40" t="s">
+        <v>129</v>
+      </c>
+      <c r="F40" t="s">
         <v>130</v>
-      </c>
-      <c r="F40" t="s">
-        <v>131</v>
       </c>
       <c r="G40" t="s">
         <v>45</v>
@@ -2260,21 +2268,21 @@
       <c r="A41" s="17">
         <v>35</v>
       </c>
-      <c r="B41" s="23" t="s">
-        <v>88</v>
-      </c>
-      <c r="C41" s="24"/>
+      <c r="B41" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="C41" s="23"/>
       <c r="D41" s="17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E41" t="s">
-        <v>132</v>
+        <v>154</v>
       </c>
       <c r="F41" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="G41" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H41" t="s">
         <v>49</v>
@@ -2284,21 +2292,21 @@
       <c r="A42" s="17">
         <v>36</v>
       </c>
-      <c r="B42" s="23" t="s">
-        <v>88</v>
-      </c>
-      <c r="C42" s="24"/>
+      <c r="B42" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="C42" s="23"/>
       <c r="D42" s="17">
         <v>3</v>
       </c>
       <c r="E42" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F42" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="G42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H42" t="s">
         <v>46</v>
@@ -2308,21 +2316,21 @@
       <c r="A43" s="17">
         <v>37</v>
       </c>
-      <c r="B43" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C43" s="24"/>
+      <c r="B43" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C43" s="23"/>
       <c r="D43" s="17">
         <v>1</v>
       </c>
       <c r="E43" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F43" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G43" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H43" t="s">
         <v>46</v>
@@ -2332,77 +2340,77 @@
       <c r="A44" s="17">
         <v>38</v>
       </c>
-      <c r="B44" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C44" s="24"/>
+      <c r="B44" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C44" s="23"/>
       <c r="D44" s="17">
         <v>1</v>
       </c>
       <c r="E44" t="s">
+        <v>136</v>
+      </c>
+      <c r="F44" t="s">
+        <v>137</v>
+      </c>
+      <c r="G44" t="s">
         <v>138</v>
       </c>
-      <c r="F44" t="s">
+      <c r="H44" t="s">
         <v>139</v>
-      </c>
-      <c r="G44" t="s">
-        <v>140</v>
-      </c>
-      <c r="H44" t="s">
-        <v>141</v>
       </c>
       <c r="K44" s="5"/>
       <c r="L44" s="5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="45" spans="1:12" ht="18.75" customHeight="1">
       <c r="A45" s="17">
         <v>39</v>
       </c>
-      <c r="B45" s="23" t="s">
-        <v>88</v>
-      </c>
-      <c r="C45" s="24"/>
+      <c r="B45" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="C45" s="23"/>
       <c r="D45" s="17">
         <v>1</v>
       </c>
       <c r="E45" t="s">
+        <v>141</v>
+      </c>
+      <c r="F45" t="s">
+        <v>142</v>
+      </c>
+      <c r="G45" t="s">
+        <v>120</v>
+      </c>
+      <c r="H45" t="s">
         <v>143</v>
       </c>
-      <c r="F45" t="s">
+      <c r="K45" s="40"/>
+      <c r="L45" s="5" t="s">
         <v>144</v>
-      </c>
-      <c r="G45" t="s">
-        <v>121</v>
-      </c>
-      <c r="H45" t="s">
-        <v>145</v>
-      </c>
-      <c r="K45" s="41"/>
-      <c r="L45" s="5" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="46" spans="1:12" ht="18.75" customHeight="1">
       <c r="A46" s="17">
         <v>40</v>
       </c>
-      <c r="B46" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C46" s="24"/>
+      <c r="B46" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C46" s="23"/>
       <c r="D46" s="17">
         <v>1</v>
       </c>
       <c r="E46" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F46" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="G46" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H46" t="s">
         <v>46</v>
@@ -2412,55 +2420,55 @@
       <c r="A47" s="17">
         <v>41</v>
       </c>
-      <c r="B47" s="23" t="s">
-        <v>88</v>
-      </c>
-      <c r="C47" s="24" t="s">
+      <c r="B47" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="C47" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="D47" s="17">
+        <v>1</v>
+      </c>
+      <c r="E47" t="s">
+        <v>148</v>
+      </c>
+      <c r="F47" t="s">
         <v>149</v>
       </c>
-      <c r="D47" s="17">
-        <v>1</v>
-      </c>
-      <c r="E47" t="s">
+      <c r="G47" t="s">
+        <v>149</v>
+      </c>
+      <c r="H47" t="s">
         <v>150</v>
       </c>
-      <c r="F47" t="s">
+      <c r="L47" s="5" t="s">
         <v>151</v>
-      </c>
-      <c r="G47" t="s">
-        <v>151</v>
-      </c>
-      <c r="H47" t="s">
-        <v>152</v>
-      </c>
-      <c r="L47" s="5" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="48" spans="1:12" ht="18.75" customHeight="1">
       <c r="A48" s="17">
         <v>42</v>
       </c>
-      <c r="B48" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C48" s="24" t="s">
-        <v>149</v>
+      <c r="B48" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C48" s="23" t="s">
+        <v>147</v>
       </c>
       <c r="D48" s="17">
         <v>2</v>
       </c>
       <c r="E48" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F48" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G48" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H48" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -2550,7 +2558,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="30">
+    <row r="7" spans="1:4">
       <c r="A7" s="17">
         <v>4</v>
       </c>
@@ -2676,8 +2684,19 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="18.75" customHeight="1">
-      <c r="B16" s="21"/>
+    <row r="16" spans="1:4" ht="30">
+      <c r="A16" s="12">
+        <v>13</v>
+      </c>
+      <c r="B16" s="27">
+        <v>45553</v>
+      </c>
+      <c r="C16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>156</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2697,11 +2716,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" customHeight="1">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
     </row>
     <row r="2" spans="1:3" ht="18.75" customHeight="1">
       <c r="A2" s="1" t="s">

</xml_diff>

<commit_message>
Hot Fix Pull up DCDC, Fix Bom CPU
Se incluyeron como futura feature. Dieron problemas de montaje y a la hora de testearse insitu. Se pasan a no montar.
En la CPU se corrije un error por el que no aparecia R22 (pull-down Enable LDO)
</commit_message>
<xml_diff>
--- a/02.HARDWARE/V2-ROVER R-1/02.BOM/BATT_DCDC.xlsx
+++ b/02.HARDWARE/V2-ROVER R-1/02.BOM/BATT_DCDC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Team Dropbox\JRODRIGUEZ\Repositorios\01.Rover\02.HARDWARE\V2-ROVER R-1\02.BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D61A479-A0A7-4DBE-80E7-D86E1F0664B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE904247-FEB7-420B-9FD5-8D90ED26C4C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BATT_DCDC" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="160">
   <si>
     <t>Document property of:</t>
   </si>
@@ -511,9 +511,6 @@
     <t>20R</t>
   </si>
   <si>
-    <t>R7,R21,R22</t>
-  </si>
-  <si>
     <t>C2, C5, C6,C8 C24,C11</t>
   </si>
   <si>
@@ -526,6 +523,19 @@
 Se añade a la posicion 35 el part R21 se cambia la cantidad de 1 a 2
 Se elimina la posicion 8 con el part R10.
 Se añade a la posicion 36 el part R10. Aumenta la cantidad de 2 a 3.</t>
+  </si>
+  <si>
+    <t>NI</t>
+  </si>
+  <si>
+    <t>R21,R22</t>
+  </si>
+  <si>
+    <t>R7</t>
+  </si>
+  <si>
+    <t>Se añade la posicion 43 con los part 21 y R22 de valor 4k2 con NO MONTAR
+Se eliminan de la posicion 35 los par R21 y R22, se cambia la cantidad de 3 a 1</t>
   </si>
 </sst>
 </file>
@@ -953,6 +963,9 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="14" fontId="12" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -969,9 +982,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -997,8 +1007,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A6:L48" totalsRowShown="0">
-  <autoFilter ref="A6:L48" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A6:L49" totalsRowShown="0">
+  <autoFilter ref="A6:L49" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Position"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="NEW" dataDxfId="0"/>
@@ -1305,7 +1315,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.42578125" style="21" bestFit="1" customWidth="1"/>
@@ -1331,7 +1341,7 @@
       </c>
       <c r="B2" s="25">
         <f>MAX(_HISTORY!A4:A55)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" s="26"/>
     </row>
@@ -1341,20 +1351,20 @@
       </c>
       <c r="B3" s="27">
         <f>VLOOKUP(B2,_HISTORY!A3:D100,2)</f>
-        <v>45553</v>
+        <v>45700</v>
       </c>
       <c r="C3" s="27"/>
       <c r="D3" s="28"/>
       <c r="E3" s="29"/>
     </row>
     <row r="4" spans="1:12" ht="30" customHeight="1">
-      <c r="B4" s="44" t="s">
+      <c r="B4" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="45"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="47"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="48"/>
     </row>
     <row r="5" spans="1:12" ht="30.75" customHeight="1">
       <c r="B5" s="30"/>
@@ -1502,14 +1512,14 @@
         <v>5</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>86</v>
+        <v>41</v>
       </c>
       <c r="C11" s="23"/>
       <c r="D11" s="17">
         <v>6</v>
       </c>
       <c r="E11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F11" t="s">
         <v>54</v>
@@ -1804,7 +1814,7 @@
         <v>16</v>
       </c>
       <c r="B22" s="43" t="s">
-        <v>86</v>
+        <v>41</v>
       </c>
       <c r="C22" s="38"/>
       <c r="D22" s="39" t="s">
@@ -2286,10 +2296,10 @@
       </c>
       <c r="C41" s="23"/>
       <c r="D41" s="17">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E41" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="F41" t="s">
         <v>130</v>
@@ -2382,7 +2392,7 @@
         <v>39</v>
       </c>
       <c r="B45" s="22" t="s">
-        <v>86</v>
+        <v>41</v>
       </c>
       <c r="C45" s="23"/>
       <c r="D45" s="17">
@@ -2401,7 +2411,7 @@
         <v>142</v>
       </c>
       <c r="K45" s="40"/>
-      <c r="L45" s="50" t="s">
+      <c r="L45" s="44" t="s">
         <v>143</v>
       </c>
     </row>
@@ -2434,7 +2444,7 @@
         <v>41</v>
       </c>
       <c r="B47" s="22" t="s">
-        <v>86</v>
+        <v>156</v>
       </c>
       <c r="C47" s="23" t="s">
         <v>146</v>
@@ -2482,6 +2492,32 @@
       </c>
       <c r="H48" t="s">
         <v>115</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49" s="21">
+        <v>43</v>
+      </c>
+      <c r="B49" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="C49" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="D49" s="21">
+        <v>2</v>
+      </c>
+      <c r="E49" t="s">
+        <v>157</v>
+      </c>
+      <c r="F49" t="s">
+        <v>130</v>
+      </c>
+      <c r="G49" t="s">
+        <v>85</v>
+      </c>
+      <c r="H49" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2503,13 +2539,13 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.5703125" style="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.5703125" style="10" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="65.42578125" style="11" customWidth="1"/>
+    <col min="4" max="4" width="133.85546875" style="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18.75" customHeight="1">
@@ -2697,7 +2733,7 @@
         <v>14</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="30">
@@ -2711,7 +2747,21 @@
         <v>14</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="30">
+      <c r="A17" s="12">
+        <v>14</v>
+      </c>
+      <c r="B17" s="10">
+        <v>45700</v>
+      </c>
+      <c r="C17" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -2732,11 +2782,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" customHeight="1">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
     </row>
     <row r="2" spans="1:3" ht="18.75" customHeight="1">
       <c r="A2" s="1" t="s">

</xml_diff>